<commit_message>
Added new plots to compare deformation zones, still working on graphically showing breakup region. >20% region not refined.
</commit_message>
<xml_diff>
--- a/We-Oh Tables 1995.xlsx
+++ b/We-Oh Tables 1995.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gtvault-my.sharepoint.com/personal/adharmasanam3_gatech_edu/Documents/0 - Research OEF/Particle Modeling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="248" documentId="8_{D1F243AE-EEDB-446F-9C32-BDD84A68E908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24BAC9D4-9BCA-44D1-AE6B-BC1F61157599}"/>
+  <xr:revisionPtr revIDLastSave="261" documentId="8_{D1F243AE-EEDB-446F-9C32-BDD84A68E908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C249044-38F6-4D6A-9166-58BCE74F7D82}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="We-Oh" sheetId="1" r:id="rId1"/>
@@ -274,18 +274,6 @@
     <t>All Breakup</t>
   </si>
   <si>
-    <t>&lt;5%</t>
-  </si>
-  <si>
-    <t>5%&lt; x &lt;10%</t>
-  </si>
-  <si>
-    <t>10%&lt; x &lt;20%</t>
-  </si>
-  <si>
-    <t>&gt;20%</t>
-  </si>
-  <si>
     <t>TAB</t>
   </si>
   <si>
@@ -293,6 +281,18 @@
   </si>
   <si>
     <t>Hsiang &amp; Faeth (1995)</t>
+  </si>
+  <si>
+    <t>Deformation &lt;5%</t>
+  </si>
+  <si>
+    <t>5%&lt; Deformation &lt;10%</t>
+  </si>
+  <si>
+    <t>10%&lt; Deformation &lt;20%</t>
+  </si>
+  <si>
+    <t>Deformation &gt;20%</t>
   </si>
 </sst>
 </file>
@@ -406,6 +406,12 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -417,12 +423,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7737,7 +7737,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&lt;5%</c:v>
+                  <c:v>Deformation &lt;5%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -7829,7 +7829,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5%&lt; x &lt;10%</c:v>
+                  <c:v>5%&lt; Deformation &lt;10%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -7921,7 +7921,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>10%&lt; x &lt;20%</c:v>
+                  <c:v>10%&lt; Deformation &lt;20%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -8013,7 +8013,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&gt;20%</c:v>
+                  <c:v>Deformation &gt;20%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -8762,7 +8762,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&lt;5%</c:v>
+                  <c:v>Deformation &lt;5%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -8854,7 +8854,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&gt;20%</c:v>
+                  <c:v>Deformation &gt;20%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -9579,7 +9579,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&lt;5%</c:v>
+                  <c:v>Deformation &lt;5%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -9648,7 +9648,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&gt;20%</c:v>
+                  <c:v>Deformation &gt;20%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -10251,7 +10251,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&lt;5%</c:v>
+                  <c:v>Deformation &lt;5%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -10343,7 +10343,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&gt;20%</c:v>
+                  <c:v>Deformation &gt;20%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -11088,7 +11088,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&lt;5%</c:v>
+                  <c:v>Deformation &lt;5%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -11180,7 +11180,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5%&lt; x &lt;10%</c:v>
+                  <c:v>5%&lt; Deformation &lt;10%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -11272,7 +11272,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>10%&lt; x &lt;20%</c:v>
+                  <c:v>10%&lt; Deformation &lt;20%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -11364,7 +11364,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&gt;20%</c:v>
+                  <c:v>Deformation &gt;20%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -12113,7 +12113,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&lt;5%</c:v>
+                  <c:v>Deformation &lt;5%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -12205,7 +12205,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5%&lt; x &lt;10%</c:v>
+                  <c:v>5%&lt; Deformation &lt;10%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -12297,7 +12297,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>10%&lt; x &lt;20%</c:v>
+                  <c:v>10%&lt; Deformation &lt;20%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -12389,7 +12389,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>&gt;20%</c:v>
+                  <c:v>Deformation &gt;20%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -18791,13 +18791,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="M1" s="5" t="s">
@@ -19622,14 +19622,14 @@
       </c>
     </row>
     <row r="25" spans="7:20" x14ac:dyDescent="0.45">
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="21"/>
+      <c r="K25" s="21"/>
+      <c r="L25" s="21"/>
       <c r="M25" s="4">
         <v>4</v>
       </c>
@@ -19659,14 +19659,14 @@
       </c>
     </row>
     <row r="26" spans="7:20" x14ac:dyDescent="0.45">
-      <c r="G26" s="19" t="s">
+      <c r="G26" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
-      <c r="J26" s="19"/>
-      <c r="K26" s="19"/>
-      <c r="L26" s="19"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
+      <c r="K26" s="21"/>
+      <c r="L26" s="21"/>
       <c r="M26" s="4">
         <v>6</v>
       </c>
@@ -19696,14 +19696,14 @@
       </c>
     </row>
     <row r="27" spans="7:20" x14ac:dyDescent="0.45">
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
-      <c r="J27" s="19"/>
-      <c r="K27" s="19"/>
-      <c r="L27" s="19"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="21"/>
+      <c r="L27" s="21"/>
       <c r="M27" s="4">
         <v>8</v>
       </c>
@@ -20175,23 +20175,23 @@
         <v>0.1</v>
       </c>
       <c r="O43">
-        <f t="shared" ref="O4:O52" si="8">SQRT(M43)/N43</f>
+        <f t="shared" ref="O43:O52" si="8">SQRT(M43)/N43</f>
         <v>24.494897427831777</v>
       </c>
       <c r="P43" s="8">
-        <f t="shared" ref="P4:P52" si="9">($C$9^2)/($C$5*$C$7*(N43^2))</f>
+        <f t="shared" ref="P43:P52" si="9">($C$9^2)/($C$5*$C$7*(N43^2))</f>
         <v>1.1322611903507131E-6</v>
       </c>
       <c r="Q43" s="7">
-        <f t="shared" ref="Q4:Q52" si="10">SQRT(M43*$C$7/(P43*$C$4))</f>
+        <f t="shared" ref="Q43:Q52" si="10">SQRT(M43*$C$7/(P43*$C$4))</f>
         <v>563.86863735038412</v>
       </c>
       <c r="S43" s="4">
-        <f t="shared" ref="S4:S52" si="11">$C$4*(Q43^2)*P43/$C$7</f>
+        <f t="shared" ref="S43:S52" si="11">$C$4*(Q43^2)*P43/$C$7</f>
         <v>6</v>
       </c>
       <c r="T43">
-        <f t="shared" ref="T4:T52" si="12">$C$9/SQRT($C$5*P43*$C$7)</f>
+        <f t="shared" ref="T43:T52" si="12">$C$9/SQRT($C$5*P43*$C$7)</f>
         <v>0.1</v>
       </c>
     </row>
@@ -20484,17 +20484,17 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" s="4"/>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" s="12" t="s">
@@ -20776,17 +20776,17 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A14" s="4"/>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A15" s="12" t="s">
@@ -21112,11 +21112,11 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -21146,18 +21146,18 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="4"/>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="12" t="s">
@@ -21167,16 +21167,16 @@
         <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G3" t="s">
         <v>45</v>
@@ -21196,7 +21196,7 @@
         <v>1E-3</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C4" s="14">
         <v>0.38</v>
@@ -21228,7 +21228,7 @@
         <v>1E-3</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C5" s="16">
         <v>0.3</v>
@@ -21260,7 +21260,7 @@
         <v>1E-3</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C6">
         <v>0.3</v>
@@ -21292,7 +21292,7 @@
         <v>0.01</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C7" s="14">
         <v>0.38</v>
@@ -21324,7 +21324,7 @@
         <v>0.01</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C8" s="16">
         <v>0.3</v>
@@ -21356,7 +21356,7 @@
         <v>0.01</v>
       </c>
       <c r="B9" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C9">
         <v>0.3</v>
@@ -21388,7 +21388,7 @@
         <v>0.1</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C10" s="14">
         <v>0.38</v>
@@ -21420,7 +21420,7 @@
         <v>0.1</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C11" s="16">
         <v>0.3</v>
@@ -21452,7 +21452,7 @@
         <v>0.1</v>
       </c>
       <c r="B12" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C12">
         <v>0.3</v>
@@ -21484,18 +21484,18 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" s="4"/>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" s="12" t="s">
@@ -21505,16 +21505,16 @@
         <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F15" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G15" t="s">
         <v>45</v>
@@ -21534,22 +21534,22 @@
         <v>1E-3</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C16" s="14">
-        <f>C4</f>
+        <f t="shared" ref="C16:C24" si="0">C4</f>
         <v>0.38</v>
       </c>
       <c r="D16" s="14">
-        <f t="shared" ref="C16:F16" si="0">D4-C4</f>
+        <f t="shared" ref="D16:F16" si="1">D4-C4</f>
         <v>0.62</v>
       </c>
       <c r="E16" s="14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.1000000000000001</v>
       </c>
       <c r="F16" s="14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.89999999999999991</v>
       </c>
       <c r="G16" s="14">
@@ -21557,11 +21557,11 @@
         <v>8</v>
       </c>
       <c r="H16" s="14">
-        <f t="shared" ref="H16:I16" si="1">H4-G4</f>
+        <f t="shared" ref="H16:I16" si="2">H4-G4</f>
         <v>24</v>
       </c>
       <c r="I16" s="14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>45</v>
       </c>
       <c r="J16" s="14">
@@ -21574,22 +21574,22 @@
         <v>1E-3</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C17" s="16">
-        <f>C5</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D17" s="16">
-        <f t="shared" ref="C17:F22" si="2">D5-C5</f>
+        <f t="shared" ref="D17:F22" si="3">D5-C5</f>
         <v>0.39999999999999997</v>
       </c>
       <c r="E17" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.8</v>
       </c>
       <c r="F17" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G17" s="16">
@@ -21597,15 +21597,15 @@
         <v>3.5</v>
       </c>
       <c r="H17" s="16">
-        <f t="shared" ref="G17:J17" si="3">H5-G5</f>
+        <f t="shared" ref="H17:J17" si="4">H5-G5</f>
         <v>0</v>
       </c>
       <c r="I17" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J17" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>995</v>
       </c>
     </row>
@@ -21614,38 +21614,38 @@
         <v>1E-3</v>
       </c>
       <c r="B18" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C18">
-        <f>C6</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.39999999999999997</v>
       </c>
       <c r="E18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.8</v>
       </c>
       <c r="F18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G18">
-        <f t="shared" ref="G18:J18" si="4">G6-F6</f>
+        <f t="shared" ref="G18:J18" si="5">G6-F6</f>
         <v>5.5</v>
       </c>
       <c r="H18">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>63</v>
       </c>
       <c r="I18">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>230</v>
       </c>
       <c r="J18">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>700</v>
       </c>
     </row>
@@ -21654,38 +21654,38 @@
         <v>0.01</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C19" s="14">
-        <f>C7</f>
+        <f t="shared" si="0"/>
         <v>0.38</v>
       </c>
       <c r="D19" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.62</v>
       </c>
       <c r="E19" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1000000000000001</v>
       </c>
       <c r="F19" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.89999999999999991</v>
       </c>
       <c r="G19" s="14">
-        <f t="shared" ref="G19:J19" si="5">G7-F7</f>
+        <f t="shared" ref="G19:J19" si="6">G7-F7</f>
         <v>8</v>
       </c>
       <c r="H19" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>24</v>
       </c>
       <c r="I19" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>45</v>
       </c>
       <c r="J19" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>920</v>
       </c>
     </row>
@@ -21694,38 +21694,38 @@
         <v>0.01</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C20" s="16">
-        <f>C8</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D20" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.39999999999999997</v>
       </c>
       <c r="E20" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.8</v>
       </c>
       <c r="F20" s="16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G20" s="16">
-        <f t="shared" ref="G20:J20" si="6">G8-F8</f>
+        <f t="shared" ref="G20:J20" si="7">G8-F8</f>
         <v>3.5</v>
       </c>
       <c r="H20" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="I20" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="J20" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>995</v>
       </c>
     </row>
@@ -21734,38 +21734,38 @@
         <v>0.01</v>
       </c>
       <c r="B21" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C21">
-        <f>C9</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.39999999999999997</v>
       </c>
       <c r="E21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.8</v>
       </c>
       <c r="F21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G21">
-        <f t="shared" ref="G21:J21" si="7">G9-F9</f>
+        <f t="shared" ref="G21:J21" si="8">G9-F9</f>
         <v>5.5</v>
       </c>
       <c r="H21">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>63</v>
       </c>
       <c r="I21">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>230</v>
       </c>
       <c r="J21">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>700</v>
       </c>
     </row>
@@ -21774,38 +21774,38 @@
         <v>0.1</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C22" s="14">
-        <f>C10</f>
+        <f t="shared" si="0"/>
         <v>0.38</v>
       </c>
       <c r="D22" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.62</v>
       </c>
       <c r="E22" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1000000000000001</v>
       </c>
       <c r="F22" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.9</v>
       </c>
       <c r="G22" s="14">
-        <f t="shared" ref="G22:J22" si="8">G10-F10</f>
+        <f t="shared" ref="G22:J22" si="9">G10-F10</f>
         <v>6</v>
       </c>
       <c r="H22" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>26</v>
       </c>
       <c r="I22" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>43</v>
       </c>
       <c r="J22" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>920</v>
       </c>
     </row>
@@ -21814,22 +21814,22 @@
         <v>0.1</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C23" s="16">
-        <f>C11</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D23" s="16">
-        <f t="shared" ref="C23:F24" si="9">D11-C11</f>
+        <f t="shared" ref="D23:F24" si="10">D11-C11</f>
         <v>0.39999999999999997</v>
       </c>
       <c r="E23" s="16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.8</v>
       </c>
       <c r="F23" s="16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1.5</v>
       </c>
       <c r="G23" s="16">
@@ -21837,15 +21837,15 @@
         <v>2</v>
       </c>
       <c r="H23" s="16">
-        <f t="shared" ref="H23:J23" si="10">H11-G11</f>
+        <f t="shared" ref="H23:J23" si="11">H11-G11</f>
         <v>0</v>
       </c>
       <c r="I23" s="16">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="J23" s="16">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>995</v>
       </c>
     </row>
@@ -21854,38 +21854,38 @@
         <v>0.1</v>
       </c>
       <c r="B24" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C24">
-        <f>C12</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.39999999999999997</v>
       </c>
       <c r="E24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.8</v>
       </c>
       <c r="F24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1.5</v>
       </c>
       <c r="G24">
-        <f t="shared" ref="G24:J24" si="11">G12-F12</f>
+        <f t="shared" ref="G24:J24" si="12">G12-F12</f>
         <v>4</v>
       </c>
       <c r="H24">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>63</v>
       </c>
       <c r="I24">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>230</v>
       </c>
       <c r="J24">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>700</v>
       </c>
     </row>
@@ -21920,11 +21920,11 @@
       <c r="B1" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
@@ -21984,7 +21984,7 @@
         <f>10^-3</f>
         <v>1E-3</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="17">
         <v>5</v>
       </c>
       <c r="H3">
@@ -22008,7 +22008,7 @@
         <f>10^-3</f>
         <v>1E-3</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="17">
         <v>1</v>
       </c>
       <c r="H4">
@@ -22032,7 +22032,7 @@
         <f t="shared" ref="E5:E19" si="0">10^-3</f>
         <v>1E-3</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="17">
         <v>1</v>
       </c>
       <c r="H5">
@@ -22056,7 +22056,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="17">
         <v>2</v>
       </c>
       <c r="H6">
@@ -22080,7 +22080,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="17">
         <v>2</v>
       </c>
       <c r="H7">
@@ -22104,7 +22104,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F8" s="21" t="s">
+      <c r="F8" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H8">
@@ -22128,7 +22128,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F9" s="21" t="s">
+      <c r="F9" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H9">
@@ -22146,7 +22146,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F10" s="21" t="s">
+      <c r="F10" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H10">
@@ -22164,7 +22164,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H11">
@@ -22182,7 +22182,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F12" s="21" t="s">
+      <c r="F12" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H12">
@@ -22200,7 +22200,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F13" s="21" t="s">
+      <c r="F13" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H13">
@@ -22218,7 +22218,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H14">
@@ -22236,7 +22236,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F15" s="21" t="s">
+      <c r="F15" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H15">
@@ -22254,7 +22254,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F16" s="21" t="s">
+      <c r="F16" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H16">
@@ -22272,7 +22272,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="F17" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H17">
@@ -22290,7 +22290,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="F18" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H18">
@@ -22308,7 +22308,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F19" s="21" t="s">
+      <c r="F19" s="17" t="s">
         <v>74</v>
       </c>
       <c r="H19">
@@ -22326,7 +22326,7 @@
         <f>10^-3</f>
         <v>1E-3</v>
       </c>
-      <c r="F20" s="21">
+      <c r="F20" s="17">
         <v>5</v>
       </c>
       <c r="H20">
@@ -22344,7 +22344,7 @@
         <f>10^-2</f>
         <v>0.01</v>
       </c>
-      <c r="F21" s="21">
+      <c r="F21" s="17">
         <v>1</v>
       </c>
       <c r="H21">
@@ -22362,7 +22362,7 @@
         <f t="shared" ref="E22:E36" si="1">10^-2</f>
         <v>0.01</v>
       </c>
-      <c r="F22" s="21">
+      <c r="F22" s="17">
         <v>1</v>
       </c>
       <c r="H22">
@@ -22380,7 +22380,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F23" s="21">
+      <c r="F23" s="17">
         <v>2</v>
       </c>
       <c r="H23">
@@ -22398,7 +22398,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F24" s="21">
+      <c r="F24" s="17">
         <v>2</v>
       </c>
       <c r="H24">
@@ -22416,7 +22416,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F25" s="21" t="s">
+      <c r="F25" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H25">
@@ -22434,7 +22434,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F26" s="21" t="s">
+      <c r="F26" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H26">
@@ -22452,7 +22452,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F27" s="21" t="s">
+      <c r="F27" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H27">
@@ -22470,7 +22470,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F28" s="21" t="s">
+      <c r="F28" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H28">
@@ -22488,7 +22488,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F29" s="21" t="s">
+      <c r="F29" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H29">
@@ -22506,7 +22506,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F30" s="21" t="s">
+      <c r="F30" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H30">
@@ -22524,7 +22524,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F31" s="21" t="s">
+      <c r="F31" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H31">
@@ -22542,7 +22542,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F32" s="21" t="s">
+      <c r="F32" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H32">
@@ -22560,7 +22560,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F33" s="21" t="s">
+      <c r="F33" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H33">
@@ -22578,7 +22578,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F34" s="21" t="s">
+      <c r="F34" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H34">
@@ -22596,7 +22596,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F35" s="21" t="s">
+      <c r="F35" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H35">
@@ -22614,7 +22614,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F36" s="21" t="s">
+      <c r="F36" s="17" t="s">
         <v>74</v>
       </c>
       <c r="H36">
@@ -22631,7 +22631,7 @@
       <c r="E37">
         <v>0.1</v>
       </c>
-      <c r="F37" s="21">
+      <c r="F37" s="17">
         <v>5</v>
       </c>
       <c r="H37">
@@ -22649,7 +22649,7 @@
         <f>10^-1</f>
         <v>0.1</v>
       </c>
-      <c r="F38" s="21">
+      <c r="F38" s="17">
         <v>1</v>
       </c>
       <c r="H38">
@@ -22667,7 +22667,7 @@
         <f t="shared" ref="E39:E53" si="2">10^-1</f>
         <v>0.1</v>
       </c>
-      <c r="F39" s="21">
+      <c r="F39" s="17">
         <v>1</v>
       </c>
       <c r="H39">
@@ -22685,7 +22685,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F40" s="21">
+      <c r="F40" s="17">
         <v>2</v>
       </c>
       <c r="H40">
@@ -22703,7 +22703,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F41" s="21">
+      <c r="F41" s="17">
         <v>2</v>
       </c>
       <c r="H41">
@@ -22721,7 +22721,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F42" s="21" t="s">
+      <c r="F42" s="17" t="s">
         <v>75</v>
       </c>
       <c r="H42">
@@ -22739,7 +22739,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F43" s="21" t="s">
+      <c r="F43" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H43">
@@ -22757,7 +22757,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F44" s="21" t="s">
+      <c r="F44" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H44">
@@ -22775,7 +22775,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F45" s="21" t="s">
+      <c r="F45" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H45">
@@ -22793,7 +22793,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F46" s="21" t="s">
+      <c r="F46" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H46">
@@ -22811,7 +22811,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F47" s="21" t="s">
+      <c r="F47" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H47">
@@ -22829,7 +22829,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F48" s="21" t="s">
+      <c r="F48" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H48">
@@ -22847,7 +22847,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F49" s="21" t="s">
+      <c r="F49" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H49">
@@ -22865,7 +22865,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F50" s="21" t="s">
+      <c r="F50" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H50">
@@ -22883,7 +22883,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F51" s="21" t="s">
+      <c r="F51" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H51">
@@ -22901,7 +22901,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F52" s="21" t="s">
+      <c r="F52" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H52">
@@ -22919,7 +22919,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F53" s="21" t="s">
+      <c r="F53" s="17" t="s">
         <v>74</v>
       </c>
       <c r="H53">
@@ -22959,11 +22959,11 @@
       <c r="B1" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
@@ -23017,7 +23017,7 @@
         <f>10^-3</f>
         <v>1E-3</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="17">
         <v>5</v>
       </c>
       <c r="H3">
@@ -23041,7 +23041,7 @@
         <f>10^-3</f>
         <v>1E-3</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="17">
         <v>1</v>
       </c>
       <c r="H4">
@@ -23065,7 +23065,7 @@
         <f t="shared" ref="E5:E19" si="0">10^-3</f>
         <v>1E-3</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="17">
         <v>1</v>
       </c>
       <c r="H5">
@@ -23089,7 +23089,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="17">
         <v>2</v>
       </c>
       <c r="H6">
@@ -23113,7 +23113,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="17">
         <v>2</v>
       </c>
       <c r="H7">
@@ -23131,7 +23131,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F8" s="21" t="s">
+      <c r="F8" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H8">
@@ -23149,7 +23149,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F9" s="21" t="s">
+      <c r="F9" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H9">
@@ -23167,7 +23167,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F10" s="21" t="s">
+      <c r="F10" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H10">
@@ -23185,7 +23185,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H11">
@@ -23203,7 +23203,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F12" s="21" t="s">
+      <c r="F12" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H12">
@@ -23221,7 +23221,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F13" s="21" t="s">
+      <c r="F13" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H13">
@@ -23239,7 +23239,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H14">
@@ -23257,7 +23257,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F15" s="21" t="s">
+      <c r="F15" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H15">
@@ -23275,7 +23275,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F16" s="21" t="s">
+      <c r="F16" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H16">
@@ -23293,7 +23293,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="F17" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H17">
@@ -23311,7 +23311,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="F18" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H18">
@@ -23329,7 +23329,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="F19" s="21" t="s">
+      <c r="F19" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H19">
@@ -23347,7 +23347,7 @@
         <f>10^-3</f>
         <v>1E-3</v>
       </c>
-      <c r="F20" s="21">
+      <c r="F20" s="17">
         <v>5</v>
       </c>
       <c r="H20">
@@ -23365,7 +23365,7 @@
         <f>10^-2</f>
         <v>0.01</v>
       </c>
-      <c r="F21" s="21">
+      <c r="F21" s="17">
         <v>1</v>
       </c>
       <c r="H21">
@@ -23383,7 +23383,7 @@
         <f t="shared" ref="E22:E36" si="1">10^-2</f>
         <v>0.01</v>
       </c>
-      <c r="F22" s="21">
+      <c r="F22" s="17">
         <v>1</v>
       </c>
       <c r="H22">
@@ -23401,7 +23401,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F23" s="21">
+      <c r="F23" s="17">
         <v>2</v>
       </c>
       <c r="H23">
@@ -23419,7 +23419,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F24" s="21">
+      <c r="F24" s="17">
         <v>2</v>
       </c>
       <c r="H24">
@@ -23437,7 +23437,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F25" s="21" t="s">
+      <c r="F25" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H25">
@@ -23455,7 +23455,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F26" s="21" t="s">
+      <c r="F26" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H26">
@@ -23473,7 +23473,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F27" s="21" t="s">
+      <c r="F27" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H27">
@@ -23491,7 +23491,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F28" s="21" t="s">
+      <c r="F28" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H28">
@@ -23509,7 +23509,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F29" s="21" t="s">
+      <c r="F29" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H29">
@@ -23527,7 +23527,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F30" s="21" t="s">
+      <c r="F30" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H30">
@@ -23545,7 +23545,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F31" s="21" t="s">
+      <c r="F31" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H31">
@@ -23563,7 +23563,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F32" s="21" t="s">
+      <c r="F32" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H32">
@@ -23581,7 +23581,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F33" s="21" t="s">
+      <c r="F33" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H33">
@@ -23599,7 +23599,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F34" s="21" t="s">
+      <c r="F34" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H34">
@@ -23617,7 +23617,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F35" s="21" t="s">
+      <c r="F35" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H35">
@@ -23635,7 +23635,7 @@
         <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
-      <c r="F36" s="21" t="s">
+      <c r="F36" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H36">
@@ -23652,7 +23652,7 @@
       <c r="E37">
         <v>0.1</v>
       </c>
-      <c r="F37" s="21">
+      <c r="F37" s="17">
         <v>5</v>
       </c>
       <c r="H37">
@@ -23670,7 +23670,7 @@
         <f>10^-1</f>
         <v>0.1</v>
       </c>
-      <c r="F38" s="21">
+      <c r="F38" s="17">
         <v>1</v>
       </c>
       <c r="H38">
@@ -23688,7 +23688,7 @@
         <f t="shared" ref="E39:E53" si="2">10^-1</f>
         <v>0.1</v>
       </c>
-      <c r="F39" s="21">
+      <c r="F39" s="17">
         <v>1</v>
       </c>
       <c r="H39">
@@ -23706,7 +23706,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F40" s="21">
+      <c r="F40" s="17">
         <v>2</v>
       </c>
       <c r="H40">
@@ -23724,7 +23724,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F41" s="21">
+      <c r="F41" s="17">
         <v>2</v>
       </c>
       <c r="H41">
@@ -23742,7 +23742,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F42" s="21" t="s">
+      <c r="F42" s="17" t="s">
         <v>75</v>
       </c>
       <c r="H42">
@@ -23760,7 +23760,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F43" s="21" t="s">
+      <c r="F43" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H43">
@@ -23778,7 +23778,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F44" s="21" t="s">
+      <c r="F44" s="17" t="s">
         <v>71</v>
       </c>
       <c r="H44">
@@ -23796,7 +23796,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F45" s="21" t="s">
+      <c r="F45" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H45">
@@ -23814,7 +23814,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F46" s="21" t="s">
+      <c r="F46" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H46">
@@ -23832,7 +23832,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F47" s="21" t="s">
+      <c r="F47" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H47">
@@ -23850,7 +23850,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F48" s="21" t="s">
+      <c r="F48" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H48">
@@ -23868,7 +23868,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F49" s="21" t="s">
+      <c r="F49" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H49">
@@ -23886,7 +23886,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F50" s="21" t="s">
+      <c r="F50" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H50">
@@ -23904,7 +23904,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F51" s="21" t="s">
+      <c r="F51" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H51">
@@ -23922,7 +23922,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F52" s="21" t="s">
+      <c r="F52" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H52">
@@ -23940,7 +23940,7 @@
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="F53" s="21" t="s">
+      <c r="F53" s="17" t="s">
         <v>72</v>
       </c>
       <c r="H53">
@@ -23951,59 +23951,59 @@
       </c>
     </row>
     <row r="54" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D54" s="22"/>
-      <c r="E54" s="22"/>
-      <c r="F54" s="22"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
+      <c r="F54" s="18"/>
     </row>
     <row r="55" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D55" s="22"/>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="18"/>
     </row>
     <row r="56" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D56" s="22"/>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+      <c r="F56" s="18"/>
     </row>
     <row r="57" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D57" s="22"/>
-      <c r="E57" s="22"/>
-      <c r="F57" s="22"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="18"/>
     </row>
     <row r="58" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D58" s="22"/>
-      <c r="E58" s="22"/>
-      <c r="F58" s="22"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="18"/>
     </row>
     <row r="59" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D59" s="22"/>
-      <c r="E59" s="22"/>
-      <c r="F59" s="22"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
     </row>
     <row r="60" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
     </row>
     <row r="61" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D61" s="22"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+      <c r="F61" s="18"/>
     </row>
     <row r="62" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D62" s="22"/>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="18"/>
     </row>
     <row r="63" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D63" s="22"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
+      <c r="D63" s="18"/>
+      <c r="E63" s="18"/>
+      <c r="F63" s="18"/>
     </row>
     <row r="64" spans="4:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D64" s="22"/>
-      <c r="E64" s="22"/>
-      <c r="F64" s="22"/>
+      <c r="D64" s="18"/>
+      <c r="E64" s="18"/>
+      <c r="F64" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Defined the deformation >20% region, updated breakup time graphs for delay in TAB vs ETAB
</commit_message>
<xml_diff>
--- a/We-Oh Tables 1995.xlsx
+++ b/We-Oh Tables 1995.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gtvault-my.sharepoint.com/personal/adharmasanam3_gatech_edu/Documents/0 - Research OEF/Particle Modeling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="261" documentId="8_{D1F243AE-EEDB-446F-9C32-BDD84A68E908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C249044-38F6-4D6A-9166-58BCE74F7D82}"/>
+  <xr:revisionPtr revIDLastSave="291" documentId="8_{D1F243AE-EEDB-446F-9C32-BDD84A68E908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{620BF877-D17C-4E36-867B-5095B898CA81}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,6 @@
     <sheet name="O'Rourke Deformation" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -4753,23 +4752,14 @@
                 <c:pt idx="6">
                   <c:v>4</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>6</c:v>
-                </c:pt>
                 <c:pt idx="22">
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="23">
                   <c:v>4</c:v>
                 </c:pt>
-                <c:pt idx="24">
-                  <c:v>6</c:v>
-                </c:pt>
                 <c:pt idx="40">
                   <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4985,6 +4975,9 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="51"/>
+                <c:pt idx="7">
+                  <c:v>6</c:v>
+                </c:pt>
                 <c:pt idx="8">
                   <c:v>8</c:v>
                 </c:pt>
@@ -5012,6 +5005,9 @@
                 <c:pt idx="16">
                   <c:v>400</c:v>
                 </c:pt>
+                <c:pt idx="24">
+                  <c:v>6</c:v>
+                </c:pt>
                 <c:pt idx="25">
                   <c:v>8</c:v>
                 </c:pt>
@@ -5038,6 +5034,9 @@
                 </c:pt>
                 <c:pt idx="33">
                   <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="42">
                   <c:v>8</c:v>
@@ -8174,7 +8173,7 @@
                   <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.5</c:v>
+                  <c:v>5.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5.5</c:v>
@@ -8454,7 +8453,7 @@
                   <c:v>920</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>995</c:v>
+                  <c:v>993</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>700</c:v>
@@ -8555,6 +8554,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Weber Numver</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -9015,7 +9069,7 @@
                   <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.5</c:v>
+                  <c:v>5.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5.5</c:v>
@@ -9291,7 +9345,7 @@
                   <c:v>920</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>995</c:v>
+                  <c:v>993</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>700</c:v>
@@ -9763,7 +9817,7 @@
                   <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.5</c:v>
+                  <c:v>5.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5.5</c:v>
@@ -9970,7 +10024,7 @@
                   <c:v>920</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>995</c:v>
+                  <c:v>993</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>700</c:v>
@@ -10504,7 +10558,7 @@
                   <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>4</c:v>
@@ -10780,7 +10834,7 @@
                   <c:v>920</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>995</c:v>
+                  <c:v>993</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>700</c:v>
@@ -11525,7 +11579,7 @@
                   <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.5</c:v>
+                  <c:v>5.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5.5</c:v>
@@ -11805,7 +11859,7 @@
                   <c:v>920</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>995</c:v>
+                  <c:v>993</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>700</c:v>
@@ -11906,6 +11960,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Weber Number</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -12550,7 +12659,7 @@
                   <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>4</c:v>
@@ -12830,7 +12939,7 @@
                   <c:v>920</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>995</c:v>
+                  <c:v>993</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>700</c:v>
@@ -12931,6 +13040,66 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Weber</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Number</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -21243,13 +21412,13 @@
         <v>1.5</v>
       </c>
       <c r="G5" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H5" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I5" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J5" s="16">
         <v>1000</v>
@@ -21339,13 +21508,13 @@
         <v>1.5</v>
       </c>
       <c r="G8" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H8" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I8" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J8" s="16">
         <v>1000</v>
@@ -21435,13 +21604,13 @@
         <v>3</v>
       </c>
       <c r="G11" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H11" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I11" s="16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J11" s="16">
         <v>1000</v>
@@ -21594,7 +21763,7 @@
       </c>
       <c r="G17" s="16">
         <f>G5-F5</f>
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="H17" s="16">
         <f t="shared" ref="H17:J17" si="4">H5-G5</f>
@@ -21606,7 +21775,7 @@
       </c>
       <c r="J17" s="16">
         <f t="shared" si="4"/>
-        <v>995</v>
+        <v>993</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.45">
@@ -21714,7 +21883,7 @@
       </c>
       <c r="G20" s="16">
         <f t="shared" ref="G20:J20" si="7">G8-F8</f>
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="H20" s="16">
         <f t="shared" si="7"/>
@@ -21726,7 +21895,7 @@
       </c>
       <c r="J20" s="16">
         <f t="shared" si="7"/>
-        <v>995</v>
+        <v>993</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.45">
@@ -21834,7 +22003,7 @@
       </c>
       <c r="G23" s="16">
         <f>G11-F11</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H23" s="16">
         <f t="shared" ref="H23:J23" si="11">H11-G11</f>
@@ -21846,7 +22015,7 @@
       </c>
       <c r="J23" s="16">
         <f t="shared" si="11"/>
-        <v>995</v>
+        <v>993</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.45">
@@ -23168,12 +23337,12 @@
         <v>1E-3</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H10">
         <v>1E-3</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>6</v>
       </c>
     </row>
@@ -23474,12 +23643,12 @@
         <v>0.01</v>
       </c>
       <c r="F27" s="17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H27">
         <v>0.01</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <v>6</v>
       </c>
     </row>
@@ -23779,12 +23948,12 @@
         <v>0.1</v>
       </c>
       <c r="F44" s="17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H44">
         <v>0.1</v>
       </c>
-      <c r="M44">
+      <c r="N44">
         <v>6</v>
       </c>
     </row>

</xml_diff>